<commit_message>
Login and Navigation to Invoice Page
</commit_message>
<xml_diff>
--- a/data/input/oem_list.xlsx
+++ b/data/input/oem_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Flux-yashas_working\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE0990BF-9592-4B47-9383-A12AB8F08B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92D71CF7-8841-4E1D-80D5-1F26E1D610B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>OEM</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>tomsmith</t>
+  </si>
+  <si>
+    <t>yashasyadavr@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://erp.magnitudotech.com </t>
   </si>
 </sst>
 </file>
@@ -393,10 +399,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -414,6 +420,7 @@
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{F4D898E8-47C3-4BFD-A4AB-A8BC494CCEE4}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{C53FDEDD-14A8-470E-AD37-BC12BF4A981F}"/>
+    <hyperlink ref="C2" r:id="rId3" xr:uid="{DBFD1F6B-28D4-4004-BD4E-CFA86589FD0C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>